<commit_message>
guard: autosave 2026-09-14 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-13 09:30</t>
+          <t>생성: 2026-09-14 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY676"/>
+  <dimension ref="A1:AY678"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64452,6 +64452,194 @@
         <v>929</v>
       </c>
     </row>
+    <row r="677">
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B677" s="8" t="n">
+        <v>121.5</v>
+      </c>
+      <c r="C677" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D677" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E677" s="8" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="F677" s="8" t="n">
+        <v>606</v>
+      </c>
+      <c r="G677" s="7" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H677" s="7" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="I677" s="7" t="n">
+        <v>-24.9</v>
+      </c>
+      <c r="J677" s="7" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="K677" s="7" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="L677" s="7" t="n">
+        <v>41.7</v>
+      </c>
+      <c r="M677" s="7" t="n">
+        <v>-19.2</v>
+      </c>
+      <c r="N677" s="8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="O677" s="8" t="n">
+        <v>232</v>
+      </c>
+      <c r="P677" s="8" t="n">
+        <v>1160</v>
+      </c>
+      <c r="Q677" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R677" s="8" t="n">
+        <v>1212</v>
+      </c>
+      <c r="S677" s="8" t="n">
+        <v>1181</v>
+      </c>
+      <c r="T677" s="8" t="n">
+        <v>1144</v>
+      </c>
+      <c r="U677" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="V677" s="8" t="n">
+        <v>172</v>
+      </c>
+      <c r="W677" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X677" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="Y677" s="8" t="n">
+        <v>790</v>
+      </c>
+      <c r="Z677" s="8" t="n">
+        <v>1170</v>
+      </c>
+      <c r="AD677" s="8" t="n">
+        <v>2532</v>
+      </c>
+      <c r="AE677" s="8" t="n">
+        <v>1409</v>
+      </c>
+      <c r="AM677" s="8" t="n">
+        <v>1227</v>
+      </c>
+      <c r="AN677" s="8" t="n">
+        <v>936</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B678" s="8" t="n">
+        <v>123.7</v>
+      </c>
+      <c r="C678" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D678" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E678" s="8" t="n">
+        <v>100.1</v>
+      </c>
+      <c r="F678" s="8" t="n">
+        <v>696</v>
+      </c>
+      <c r="G678" s="7" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="H678" s="7" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="I678" s="7" t="n">
+        <v>-20.5</v>
+      </c>
+      <c r="J678" s="7" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="K678" s="7" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="L678" s="7" t="n">
+        <v>60.2</v>
+      </c>
+      <c r="M678" s="7" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="N678" s="8" t="n">
+        <v>1150</v>
+      </c>
+      <c r="O678" s="8" t="n">
+        <v>182</v>
+      </c>
+      <c r="P678" s="8" t="n">
+        <v>1160</v>
+      </c>
+      <c r="Q678" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R678" s="8" t="n">
+        <v>1202</v>
+      </c>
+      <c r="S678" s="8" t="n">
+        <v>1194</v>
+      </c>
+      <c r="T678" s="8" t="n">
+        <v>1149</v>
+      </c>
+      <c r="U678" s="8" t="n">
+        <v>1085</v>
+      </c>
+      <c r="V678" s="8" t="n">
+        <v>117</v>
+      </c>
+      <c r="W678" s="8" t="n">
+        <v>1320</v>
+      </c>
+      <c r="X678" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="Y678" s="8" t="n">
+        <v>750</v>
+      </c>
+      <c r="Z678" s="8" t="n">
+        <v>1170</v>
+      </c>
+      <c r="AD678" s="8" t="n">
+        <v>2500</v>
+      </c>
+      <c r="AE678" s="8" t="n">
+        <v>1379</v>
+      </c>
+      <c r="AM678" s="8" t="n">
+        <v>1228</v>
+      </c>
+      <c r="AN678" s="8" t="n">
+        <v>939</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -64463,7 +64651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY141"/>
+  <dimension ref="A1:AY142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -86854,6 +87042,163 @@
       </c>
       <c r="AY141" s="8" t="n">
         <v>1915</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09 W2</t>
+        </is>
+      </c>
+      <c r="B142" s="8" t="n">
+        <v>116.5</v>
+      </c>
+      <c r="C142" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D142" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E142" s="8" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="F142" s="8" t="n">
+        <v>909</v>
+      </c>
+      <c r="G142" s="7" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H142" s="7" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="I142" s="7" t="n">
+        <v>-19.7</v>
+      </c>
+      <c r="J142" s="7" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="K142" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="L142" s="7" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="M142" s="7" t="n">
+        <v>-15.9</v>
+      </c>
+      <c r="N142" s="8" t="n">
+        <v>1142</v>
+      </c>
+      <c r="O142" s="8" t="n">
+        <v>233</v>
+      </c>
+      <c r="P142" s="8" t="n">
+        <v>1146</v>
+      </c>
+      <c r="Q142" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R142" s="8" t="n">
+        <v>1170</v>
+      </c>
+      <c r="S142" s="8" t="n">
+        <v>1134</v>
+      </c>
+      <c r="T142" s="8" t="n">
+        <v>1104</v>
+      </c>
+      <c r="U142" s="8" t="n">
+        <v>1077</v>
+      </c>
+      <c r="V142" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="W142" s="8" t="n">
+        <v>1318</v>
+      </c>
+      <c r="X142" s="8" t="n">
+        <v>1063</v>
+      </c>
+      <c r="Y142" s="8" t="n">
+        <v>764</v>
+      </c>
+      <c r="Z142" s="8" t="n">
+        <v>1158</v>
+      </c>
+      <c r="AA142" s="8" t="n">
+        <v>1535</v>
+      </c>
+      <c r="AB142" s="8" t="n">
+        <v>1280</v>
+      </c>
+      <c r="AC142" s="8" t="n">
+        <v>2230</v>
+      </c>
+      <c r="AD142" s="8" t="n">
+        <v>2524</v>
+      </c>
+      <c r="AE142" s="8" t="n">
+        <v>1365</v>
+      </c>
+      <c r="AF142" s="8" t="n">
+        <v>1419</v>
+      </c>
+      <c r="AG142" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="AH142" s="8" t="n">
+        <v>1570</v>
+      </c>
+      <c r="AI142" s="8" t="n">
+        <v>340</v>
+      </c>
+      <c r="AJ142" s="8" t="n">
+        <v>620</v>
+      </c>
+      <c r="AK142" s="8" t="n">
+        <v>383</v>
+      </c>
+      <c r="AL142" s="8" t="n">
+        <v>790</v>
+      </c>
+      <c r="AM142" s="8" t="n">
+        <v>1204</v>
+      </c>
+      <c r="AN142" s="8" t="n">
+        <v>922</v>
+      </c>
+      <c r="AO142" s="8" t="n">
+        <v>1105</v>
+      </c>
+      <c r="AP142" s="8" t="n">
+        <v>1110</v>
+      </c>
+      <c r="AQ142" s="8" t="n">
+        <v>1090</v>
+      </c>
+      <c r="AR142" s="8" t="n">
+        <v>1375</v>
+      </c>
+      <c r="AS142" s="8" t="n">
+        <v>1420</v>
+      </c>
+      <c r="AT142" s="8" t="n">
+        <v>2465</v>
+      </c>
+      <c r="AU142" s="8" t="n">
+        <v>2460</v>
+      </c>
+      <c r="AV142" s="8" t="n">
+        <v>1345</v>
+      </c>
+      <c r="AW142" s="8" t="n">
+        <v>1340</v>
+      </c>
+      <c r="AX142" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AY142" s="8" t="n">
+        <v>2005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-09-15 09:40
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-15 08:01</t>
+          <t>생성: 2026-09-15 09:30</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY678"/>
+  <dimension ref="A1:AY679"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64565,7 +64565,7 @@
         <v>100.1</v>
       </c>
       <c r="F678" s="8" t="n">
-        <v>696</v>
+        <v>969</v>
       </c>
       <c r="G678" s="7" t="n">
         <v>16.6</v>
@@ -64638,6 +64638,100 @@
       </c>
       <c r="AN678" s="8" t="n">
         <v>939</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B679" s="8" t="n">
+        <v>126.7</v>
+      </c>
+      <c r="C679" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D679" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E679" s="8" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="F679" s="8" t="n">
+        <v>982</v>
+      </c>
+      <c r="G679" s="7" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H679" s="7" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="I679" s="7" t="n">
+        <v>-21.2</v>
+      </c>
+      <c r="J679" s="7" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="K679" s="7" t="n">
+        <v>57.9</v>
+      </c>
+      <c r="L679" s="7" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="M679" s="7" t="n">
+        <v>-13.6</v>
+      </c>
+      <c r="N679" s="8" t="n">
+        <v>1150</v>
+      </c>
+      <c r="O679" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="P679" s="8" t="n">
+        <v>1160</v>
+      </c>
+      <c r="Q679" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R679" s="8" t="n">
+        <v>1194</v>
+      </c>
+      <c r="S679" s="8" t="n">
+        <v>1194</v>
+      </c>
+      <c r="T679" s="8" t="n">
+        <v>1163</v>
+      </c>
+      <c r="U679" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="V679" s="7" t="n">
+        <v>98</v>
+      </c>
+      <c r="W679" s="8" t="n">
+        <v>1330</v>
+      </c>
+      <c r="X679" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="Y679" s="8" t="n">
+        <v>745</v>
+      </c>
+      <c r="Z679" s="8" t="n">
+        <v>1170</v>
+      </c>
+      <c r="AD679" s="8" t="n">
+        <v>2446</v>
+      </c>
+      <c r="AE679" s="8" t="n">
+        <v>1387</v>
+      </c>
+      <c r="AM679" s="8" t="n">
+        <v>1246</v>
+      </c>
+      <c r="AN679" s="8" t="n">
+        <v>952</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guard: autosave 2026-09-16 08:10
</commit_message>
<xml_diff>
--- a/data/chem_prices.xlsx
+++ b/data/chem_prices.xlsx
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>생성: 2026-09-15 09:30</t>
+          <t>생성: 2026-09-16 08:01</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY679"/>
+  <dimension ref="A1:AY680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64732,6 +64732,100 @@
       </c>
       <c r="AN679" s="8" t="n">
         <v>952</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B680" s="8" t="n">
+        <v>127.7</v>
+      </c>
+      <c r="C680" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D680" s="7" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E680" s="8" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="F680" s="8" t="n">
+        <v>956</v>
+      </c>
+      <c r="G680" s="7" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="H680" s="7" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="I680" s="7" t="n">
+        <v>-25.2</v>
+      </c>
+      <c r="J680" s="7" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="K680" s="7" t="n">
+        <v>52.8</v>
+      </c>
+      <c r="L680" s="7" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="M680" s="7" t="n">
+        <v>-15.2</v>
+      </c>
+      <c r="N680" s="8" t="n">
+        <v>1150</v>
+      </c>
+      <c r="O680" s="8" t="n">
+        <v>194</v>
+      </c>
+      <c r="P680" s="8" t="n">
+        <v>1185</v>
+      </c>
+      <c r="Q680" s="8" t="n">
+        <v>1520</v>
+      </c>
+      <c r="R680" s="8" t="n">
+        <v>1193</v>
+      </c>
+      <c r="S680" s="8" t="n">
+        <v>1201</v>
+      </c>
+      <c r="T680" s="8" t="n">
+        <v>1188</v>
+      </c>
+      <c r="U680" s="8" t="n">
+        <v>1080</v>
+      </c>
+      <c r="V680" s="8" t="n">
+        <v>124</v>
+      </c>
+      <c r="W680" s="8" t="n">
+        <v>1330</v>
+      </c>
+      <c r="X680" s="8" t="n">
+        <v>1070</v>
+      </c>
+      <c r="Y680" s="8" t="n">
+        <v>810</v>
+      </c>
+      <c r="Z680" s="8" t="n">
+        <v>1170</v>
+      </c>
+      <c r="AD680" s="8" t="n">
+        <v>2418</v>
+      </c>
+      <c r="AE680" s="8" t="n">
+        <v>1400</v>
+      </c>
+      <c r="AM680" s="8" t="n">
+        <v>1260</v>
+      </c>
+      <c r="AN680" s="8" t="n">
+        <v>960</v>
       </c>
     </row>
   </sheetData>

</xml_diff>